<commit_message>
Restructure Excel workbook to show Calculateur sheet by default
</commit_message>
<xml_diff>
--- a/Calculateur_Mousse_Polyurethane.xlsx
+++ b/Calculateur_Mousse_Polyurethane.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grille" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculateur" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculateur" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grille" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +23,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.00 €"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,6 +77,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
@@ -101,14 +107,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-        <bgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -160,28 +166,16 @@
   <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -204,11 +198,23 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="11" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="12" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -574,6 +580,321 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Calculateur Mousse Polyuréthane (Factures &amp; Marge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1. DONNÉES DU PROJET (SAISIE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Surface Totale (Métrage)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Prix Client au m²</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>€/m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Votre Prix de Vente (Client) Total</t>
+        </is>
+      </c>
+      <c r="B6" s="7">
+        <f>B4*B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Épaisseur de mousse</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>10 cm</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>cm</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Distance de Déplacement</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Rayon ≤ 30 Km</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Choix</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Conditions Partenaire</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Oui / Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Délai de Paiement</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>30 jours (Standard)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Choix</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Majoration Sous-traitant</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2. DÉTAILS DU COÛT SOUS-TRAITANT</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Catégorie de Surface (Calculée)</t>
+        </is>
+      </c>
+      <c r="B15" s="11">
+        <f>IF(B4&lt;50, "&lt;50M2 (FORFAIT)", IF(B4&lt;100, "50-100M2 (+5%)", IF(B4&lt;150, "100-150M2 (0%)", IF(B4&lt;250, "150-250M2 (-2%)", IF(B4&lt;=400, "250-400M2 (-5%)", "&gt;400M2 (-8%)")))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Tarif de Base NESTAAN</t>
+        </is>
+      </c>
+      <c r="B16" s="12">
+        <f>INDEX(Grille!$B$3:$G$21, MATCH(B7, Grille!$A$3:$A$21, 0), MATCH(B15, Grille!$B$2:$G$2, 0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Base avec Majoration (+10%)</t>
+        </is>
+      </c>
+      <c r="B17" s="14">
+        <f>B16*(1+B11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Ajustement Rayon / Distance</t>
+        </is>
+      </c>
+      <c r="B18" s="15">
+        <f>IF(B8="Rayon de 30 à 60 Km", 1.01, IF(B8="Rayon &gt; 60 Km", 1.02, 1.00))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Ajustement Partenaire (-10%)</t>
+        </is>
+      </c>
+      <c r="B19" s="15">
+        <f>IF(B9="Oui", 0.90, 1.00)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Ajustement Escompte (-2%)</t>
+        </is>
+      </c>
+      <c r="B20" s="15">
+        <f>IF(B10="8 jours (-2%)", 0.98, 1.00)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Tarif Unitaire Final Sous-traitant</t>
+        </is>
+      </c>
+      <c r="B21" s="14">
+        <f>B17*B18*B19*B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>3. RÉSULTATS &amp; DIFFÉRENCE (MARGE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Coût Sous-traitant (A)</t>
+        </is>
+      </c>
+      <c r="B24" s="16">
+        <f>IF(B4&lt;50, B21, B21*B4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Votre Facturation Client (B)</t>
+        </is>
+      </c>
+      <c r="B25" s="17">
+        <f>B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>DIFFÉRENCE (Bénéfice B - A)</t>
+        </is>
+      </c>
+      <c r="B26" s="19">
+        <f>B25-B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Marge Bénéficiaire (%)</t>
+        </is>
+      </c>
+      <c r="B27" s="20">
+        <f>IF(B25&gt;0, B26/B25, 0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Grille!$A$3:$A$21</formula1>
+    </dataValidation>
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Rayon ≤ 30 Km,Rayon de 30 à 60 Km,Rayon &gt; 60 Km"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Oui,Non"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"30 jours (Standard),8 jours (-2%)"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -594,833 +915,518 @@
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Épaisseur</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>&gt;400M2 (-8%)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="21" t="inlineStr">
         <is>
           <t>250-400M2 (-5%)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>150-250M2 (-2%)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="21" t="inlineStr">
         <is>
           <t>100-150M2 (0%)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="21" t="inlineStr">
         <is>
           <t>50-100M2 (+5%)</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="21" t="inlineStr">
         <is>
           <t>&lt;50M2 (FORFAIT)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>5 cm</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="23" t="n">
         <v>12.23</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="23" t="n">
         <v>12.63</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="23" t="n">
         <v>13.03</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="23" t="n">
         <v>13.3</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="F3" s="23" t="n">
         <v>13.96</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="G3" s="24" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>6 cm</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="23" t="n">
         <v>13.39</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="23" t="n">
         <v>13.83</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="23" t="n">
         <v>14.26</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="23" t="n">
         <v>14.56</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="23" t="n">
         <v>15.28</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="G4" s="24" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>7 cm</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="23" t="n">
         <v>14.55</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="23" t="n">
         <v>15.02</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="23" t="n">
         <v>15.5</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="23" t="n">
         <v>15.82</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="23" t="n">
         <v>16.61</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="24" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>8 cm</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="23" t="n">
         <v>15.71</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="23" t="n">
         <v>16.22</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="23" t="n">
         <v>16.73</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="23" t="n">
         <v>17.08</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="23" t="n">
         <v>17.93</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="G6" s="24" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>9 cm</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="23" t="n">
         <v>16.87</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="23" t="n">
         <v>17.42</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="23" t="n">
         <v>17.97</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="23" t="n">
         <v>18.34</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="23" t="n">
         <v>19.25</v>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G7" s="24" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>10 cm</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="23" t="n">
         <v>18.03</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="23" t="n">
         <v>18.62</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="23" t="n">
         <v>19.2</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="23" t="n">
         <v>19.6</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="F8" s="23" t="n">
         <v>20.58</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="24" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>11 cm</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="23" t="n">
         <v>19.19</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="23" t="n">
         <v>19.81</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="23" t="n">
         <v>20.44</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="23" t="n">
         <v>20.86</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F9" s="23" t="n">
         <v>21.9</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="24" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>12 cm</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="23" t="n">
         <v>20.35</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="23" t="n">
         <v>21.01</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="23" t="n">
         <v>21.67</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="23" t="n">
         <v>22.12</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="F10" s="23" t="n">
         <v>23.22</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="G10" s="24" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>13 cm</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="23" t="n">
         <v>21.5</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="23" t="n">
         <v>22.21</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="23" t="n">
         <v>22.91</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="23" t="n">
         <v>23.38</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="F11" s="23" t="n">
         <v>24.54</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="24" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>14 cm</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="23" t="n">
         <v>22.66</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="23" t="n">
         <v>23.4</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="23" t="n">
         <v>24.14</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="23" t="n">
         <v>24.64</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="F12" s="23" t="n">
         <v>25.87</v>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="G12" s="24" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>15 cm</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="23" t="n">
         <v>23.82</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="23" t="n">
         <v>24.6</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="23" t="n">
         <v>25.38</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="23" t="n">
         <v>25.9</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F13" s="23" t="n">
         <v>27.19</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="24" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>16 cm</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="23" t="n">
         <v>24.98</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="23" t="n">
         <v>25.8</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="23" t="n">
         <v>26.61</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="23" t="n">
         <v>27.16</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="F14" s="23" t="n">
         <v>28.51</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="24" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>17 cm</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="23" t="n">
         <v>26.14</v>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="23" t="n">
         <v>26.99</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="23" t="n">
         <v>27.85</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="23" t="n">
         <v>28.42</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="F15" s="23" t="n">
         <v>29.84</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="24" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>18 cm</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" s="23" t="n">
         <v>27.3</v>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="23" t="n">
         <v>28.19</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="23" t="n">
         <v>29.08</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="23" t="n">
         <v>29.68</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="F16" s="23" t="n">
         <v>31.16</v>
       </c>
-      <c r="G16" s="5" t="n">
+      <c r="G16" s="24" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>19 cm</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="23" t="n">
         <v>28.46</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="23" t="n">
         <v>29.39</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="23" t="n">
         <v>30.32</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" s="23" t="n">
         <v>30.94</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="F17" s="23" t="n">
         <v>32.48</v>
       </c>
-      <c r="G17" s="5" t="n">
+      <c r="G17" s="24" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>20 cm</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="23" t="n">
         <v>29.62</v>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="23" t="n">
         <v>30.59</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="23" t="n">
         <v>31.55</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="23" t="n">
         <v>32.2</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="F18" s="23" t="n">
         <v>33.81</v>
       </c>
-      <c r="G18" s="5" t="n">
+      <c r="G18" s="24" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>21 cm</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="23" t="n">
         <v>30.78</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="23" t="n">
         <v>31.78</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="23" t="n">
         <v>32.79</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" s="23" t="n">
         <v>33.46</v>
       </c>
-      <c r="F19" s="4" t="n">
+      <c r="F19" s="23" t="n">
         <v>35.13</v>
       </c>
-      <c r="G19" s="5" t="n">
+      <c r="G19" s="24" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>23 cm</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n">
+      <c r="B20" s="23" t="n">
         <v>33.1</v>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="23" t="n">
         <v>34.18</v>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="D20" s="23" t="n">
         <v>35.26</v>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" s="23" t="n">
         <v>35.98</v>
       </c>
-      <c r="F20" s="4" t="n">
+      <c r="F20" s="23" t="n">
         <v>37.77</v>
       </c>
-      <c r="G20" s="5" t="n">
+      <c r="G20" s="24" t="n">
         <v>1800</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>25 cm</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n">
+      <c r="B21" s="23" t="n">
         <v>35.42</v>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="23" t="n">
         <v>36.57</v>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" s="23" t="n">
         <v>37.73</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" s="23" t="n">
         <v>38.5</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="F21" s="23" t="n">
         <v>40.42</v>
       </c>
-      <c r="G21" s="5" t="n">
+      <c r="G21" s="24" t="n">
         <v>1800</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Calculateur Mousse Polyuréthane - NESTAAN S-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>1. DONNÉES DU PROJET</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Surface Totale (Métrage)</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Prix Client au m²</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="n">
-        <v>83.33</v>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>€/m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>Votre Prix de Vente (Client)</t>
-        </is>
-      </c>
-      <c r="B6" s="11">
-        <f>B4*B5</f>
-        <v/>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Épaisseur de mousse</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>10 cm</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>cm</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Distance de Déplacement</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>Rayon ≤ 30 Km</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Choix</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>Conditions Partenaire</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Oui / Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Délai de Paiement</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>30 jours (Standard)</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Choix</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Majoration Sous-traitant</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>2. DÉTAILS DU CALCUL (SOUS-TRAITANT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>Catégorie de Surface</t>
-        </is>
-      </c>
-      <c r="B15" s="15">
-        <f>IF(B4&lt;50, "&lt;50M2 (FORFAIT)", IF(B4&lt;100, "50-100M2 (+5%)", IF(B4&lt;150, "100-150M2 (0%)", IF(B4&lt;250, "150-250M2 (-2%)", IF(B4&lt;=400, "250-400M2 (-5%)", "&gt;400M2 (-8%)")))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Tarif de Base NESTAAN</t>
-        </is>
-      </c>
-      <c r="B16" s="16">
-        <f>INDEX(Grille!$B$3:$G$21, MATCH(B7, Grille!$A$3:$A$21, 0), MATCH(B15, Grille!$B$2:$G$2, 0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Base avec Majoration</t>
-        </is>
-      </c>
-      <c r="B17" s="18">
-        <f>B16*(1+B11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Ajustement Rayon / Distance</t>
-        </is>
-      </c>
-      <c r="B18" s="19">
-        <f>IF(B8="Rayon de 30 à 60 Km", 1.01, IF(B8="Rayon &gt; 60 Km", 1.02, 1.00))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
-          <t>Ajustement Partenaire</t>
-        </is>
-      </c>
-      <c r="B19" s="19">
-        <f>IF(B9="Oui", 0.90, 1.00)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>Ajustement Escompte</t>
-        </is>
-      </c>
-      <c r="B20" s="19">
-        <f>IF(B10="8 jours (-2%)", 0.98, 1.00)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Tarif Unitaire Final Sous-traitant</t>
-        </is>
-      </c>
-      <c r="B21" s="18">
-        <f>B17*B18*B19*B20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>3. RÉSULTATS FINANCIERS</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Coût Sous-traitant Total</t>
-        </is>
-      </c>
-      <c r="B24" s="20">
-        <f>IF(B4&lt;50, B21, B21*B4)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Facturation Client</t>
-        </is>
-      </c>
-      <c r="B25" s="21">
-        <f>B6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="A26" s="22" t="inlineStr">
-        <is>
-          <t>Bénéfice Net (Différence)</t>
-        </is>
-      </c>
-      <c r="B26" s="23">
-        <f>B25-B24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Marge Bénéficiaire (%)</t>
-        </is>
-      </c>
-      <c r="B27" s="24">
-        <f>IF(B25&gt;0, B26/B25, 0)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Choix invalide" error="Votre valeur n'est pas dans la liste d'épaisseurs" promptTitle="Épaisseur" prompt="Sélectionnez l'épaisseur (ex: 10 cm)" type="list">
-      <formula1>Grille!$A$3:$A$21</formula1>
-    </dataValidation>
-    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Rayon ≤ 30 Km,Rayon de 30 à 60 Km,Rayon &gt; 60 Km"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Oui,Non"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"30 jours (Standard),8 jours (-2%)"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Improve Excel styling with larger typography, colored card blocks, and margins
</commit_message>
<xml_diff>
--- a/Calculateur_Mousse_Polyurethane.xlsx
+++ b/Calculateur_Mousse_Polyurethane.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.00 €"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,67 +32,109 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001F4E78"/>
+      <color rgb="001e293b"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001F4E78"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00334155"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="0064748B"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
+      <color rgb="00475569"/>
       <sz val="11"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="00595959"/>
-    </font>
-    <font>
-      <i val="1"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C00000"/>
+      <name val="Segoe UI"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001F4E78"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00375623"/>
+      <color rgb="00991B1B"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00991B1B"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000369A1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000369A1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00166534"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00166534"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00166534"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -101,30 +143,48 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="001e293b"/>
+        <bgColor rgb="001e293b"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-        <bgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00334155"/>
+        <bgColor rgb="00334155"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0F2FE"/>
+        <bgColor rgb="00E0F2FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+        <bgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -134,75 +194,199 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D3D3D3"/>
+        <color rgb="00CBD5E1"/>
       </left>
       <right style="thin">
-        <color rgb="00D3D3D3"/>
+        <color rgb="00CBD5E1"/>
       </right>
       <top style="thin">
-        <color rgb="00D3D3D3"/>
+        <color rgb="00CBD5E1"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D3D3D3"/>
+        <color rgb="00CBD5E1"/>
       </bottom>
     </border>
     <border>
-      <bottom style="medium">
-        <color rgb="001F4E78"/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
       </bottom>
     </border>
     <border>
       <top style="thin">
-        <color rgb="00D3D3D3"/>
+        <color rgb="00CBD5E1"/>
       </top>
       <bottom style="double">
-        <color rgb="00000000"/>
+        <color rgb="00166534"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00475569"/>
+      </left>
+      <bottom/>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="00475569"/>
+      </right>
+      <bottom/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00475569"/>
+      </left>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="00475569"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00475569"/>
+      </left>
+      <top style="medium">
+        <color rgb="00475569"/>
+      </top>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00475569"/>
+      </left>
+      <bottom style="medium">
+        <color rgb="00475569"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00475569"/>
+      </top>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00475569"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="00475569"/>
+      </right>
+      <top style="medium">
+        <color rgb="00475569"/>
+      </top>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="00475569"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="00475569"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00475569"/>
+      </left>
+      <bottom style="double">
+        <color rgb="00166534"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="00475569"/>
+      </right>
+      <bottom style="double">
+        <color rgb="00166534"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="18" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="12" fillId="5" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -580,308 +764,329 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="B2:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Calculateur Mousse Polyuréthane (Factures &amp; Marge)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>1. DONNÉES DU PROJET (SAISIE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="2" ht="45" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Calculateur Mousse Polyuréthane</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 1. DONNÉES DU PROJET (SAISIE)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Surface Totale (Métrage)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="C5" s="6" t="n">
         <v>120</v>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6" ht="28" customHeight="1">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Prix Client au m²</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="C6" s="8" t="n">
         <v>83.33</v>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>€/m²</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7" ht="28" customHeight="1">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Votre Prix de Vente (Client) Total</t>
         </is>
       </c>
-      <c r="B6" s="7">
-        <f>B4*B5</f>
+      <c r="C7" s="9">
+        <f>C5*C6</f>
         <v/>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>€</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="8" ht="28" customHeight="1">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Épaisseur de mousse</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>10 cm</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>cm</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9" ht="28" customHeight="1">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Distance de Déplacement</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Rayon ≤ 30 Km</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Choix</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="10" ht="28" customHeight="1">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Conditions Partenaire</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Oui / Non</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="11" ht="28" customHeight="1">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Délai de Paiement</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>30 jours (Standard)</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Choix</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="12" ht="28" customHeight="1">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Majoration Sous-traitant</t>
         </is>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="C12" s="12" t="n">
         <v>0.1</v>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>2. DÉTAILS DU COÛT SOUS-TRAITANT</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Catégorie de Surface (Calculée)</t>
-        </is>
-      </c>
-      <c r="B15" s="11">
-        <f>IF(B4&lt;50, "&lt;50M2 (FORFAIT)", IF(B4&lt;100, "50-100M2 (+5%)", IF(B4&lt;150, "100-150M2 (0%)", IF(B4&lt;250, "150-250M2 (-2%)", IF(B4&lt;=400, "250-400M2 (-5%)", "&gt;400M2 (-8%)")))))</f>
+    <row r="14" ht="30" customHeight="1">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 2. DÉTAILS DU COÛT SOUS-TRAITANT</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>Catégorie de Surface</t>
+        </is>
+      </c>
+      <c r="C15" s="15">
+        <f>IF(C5&lt;50, "&lt;50M2 (FORFAIT)", IF(C5&lt;100, "50-100M2 (+5%)", IF(C5&lt;150, "100-150M2 (0%)", IF(C5&lt;250, "150-250M2 (-2%)", IF(C5&lt;=400, "250-400M2 (-5%)", "&gt;400M2 (-8%)")))))</f>
         <v/>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr"/>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Tarif de Base NESTAAN</t>
         </is>
       </c>
-      <c r="B16" s="12">
-        <f>INDEX(Grille!$B$3:$G$21, MATCH(B7, Grille!$A$3:$A$21, 0), MATCH(B15, Grille!$B$2:$G$2, 0))</f>
+      <c r="C16" s="15">
+        <f>INDEX(Grille!$B$3:$G$21, MATCH(C8, Grille!$A$3:$A$21, 0), MATCH(C15, Grille!$B$2:$G$2, 0))</f>
         <v/>
       </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Base avec Majoration (+10%)</t>
-        </is>
-      </c>
-      <c r="B17" s="14">
-        <f>B16*(1+B11)</f>
+      <c r="D16" s="16" t="inlineStr"/>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Base avec Majoration</t>
+        </is>
+      </c>
+      <c r="C17" s="15">
+        <f>C16*(1+C12)</f>
         <v/>
       </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="D17" s="16" t="inlineStr"/>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Ajustement Rayon / Distance</t>
         </is>
       </c>
-      <c r="B18" s="15">
-        <f>IF(B8="Rayon de 30 à 60 Km", 1.01, IF(B8="Rayon &gt; 60 Km", 1.02, 1.00))</f>
+      <c r="C18" s="17">
+        <f>IF(C9="Rayon de 30 à 60 Km", 1.01, IF(C9="Rayon &gt; 60 Km", 1.02, 1.00))</f>
         <v/>
       </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>Ajustement Partenaire (-10%)</t>
         </is>
       </c>
-      <c r="B19" s="15">
-        <f>IF(B9="Oui", 0.90, 1.00)</f>
+      <c r="C19" s="17">
+        <f>IF(C10="Oui", 0.90, 1.00)</f>
         <v/>
       </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr"/>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Ajustement Escompte (-2%)</t>
         </is>
       </c>
-      <c r="B20" s="15">
-        <f>IF(B10="8 jours (-2%)", 0.98, 1.00)</f>
+      <c r="C20" s="17">
+        <f>IF(C11="8 jours (-2%)", 0.98, 1.00)</f>
         <v/>
       </c>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="D20" s="16" t="inlineStr"/>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Tarif Unitaire Final Sous-traitant</t>
         </is>
       </c>
-      <c r="B21" s="14">
-        <f>B17*B18*B19*B20</f>
+      <c r="C21" s="18">
+        <f>C17*C18*C19*C20</f>
         <v/>
       </c>
-    </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>3. RÉSULTATS &amp; DIFFÉRENCE (MARGE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 3. RÉSULTATS &amp; DIFFÉRENCE (MARGE)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="4" t="n"/>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>Coût Sous-traitant (A)</t>
         </is>
       </c>
-      <c r="B24" s="16">
-        <f>IF(B4&lt;50, B21, B21*B4)</f>
+      <c r="C24" s="21">
+        <f>IF(C5&lt;50, C21, C21*C5)</f>
         <v/>
       </c>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="D24" s="22" t="n"/>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t>Votre Facturation Client (B)</t>
         </is>
       </c>
-      <c r="B25" s="17">
-        <f>B6</f>
+      <c r="C25" s="24">
+        <f>C7</f>
         <v/>
       </c>
-    </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="D25" s="25" t="n"/>
+    </row>
+    <row r="26" ht="38" customHeight="1">
+      <c r="B26" s="26" t="inlineStr">
         <is>
           <t>DIFFÉRENCE (Bénéfice B - A)</t>
         </is>
       </c>
-      <c r="B26" s="19">
-        <f>B25-B24</f>
+      <c r="C26" s="27">
+        <f>C25-C24</f>
         <v/>
       </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="D26" s="28" t="n"/>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Marge Bénéficiaire (%)</t>
         </is>
       </c>
-      <c r="B27" s="20">
-        <f>IF(B25&gt;0, B26/B25, 0)</f>
+      <c r="C27" s="29">
+        <f>IF(C25&gt;0, C26/C25, 0)</f>
         <v/>
       </c>
+      <c r="D27" s="19" t="n"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B4:D4"/>
+  </mergeCells>
   <dataValidations count="4">
-    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Grille!$A$3:$A$21</formula1>
     </dataValidation>
-    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Rayon ≤ 30 Km,Rayon de 30 à 60 Km,Rayon &gt; 60 Km"</formula1>
     </dataValidation>
-    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Oui,Non"</formula1>
     </dataValidation>
-    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"30 jours (Standard),8 jours (-2%)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -908,521 +1113,521 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>Grille de Tarifs NESTAAN S-09 (Hors TVA)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="31" t="inlineStr">
         <is>
           <t>Épaisseur</t>
         </is>
       </c>
-      <c r="B2" s="21" t="inlineStr">
+      <c r="B2" s="31" t="inlineStr">
         <is>
           <t>&gt;400M2 (-8%)</t>
         </is>
       </c>
-      <c r="C2" s="21" t="inlineStr">
+      <c r="C2" s="31" t="inlineStr">
         <is>
           <t>250-400M2 (-5%)</t>
         </is>
       </c>
-      <c r="D2" s="21" t="inlineStr">
+      <c r="D2" s="31" t="inlineStr">
         <is>
           <t>150-250M2 (-2%)</t>
         </is>
       </c>
-      <c r="E2" s="21" t="inlineStr">
+      <c r="E2" s="31" t="inlineStr">
         <is>
           <t>100-150M2 (0%)</t>
         </is>
       </c>
-      <c r="F2" s="21" t="inlineStr">
+      <c r="F2" s="31" t="inlineStr">
         <is>
           <t>50-100M2 (+5%)</t>
         </is>
       </c>
-      <c r="G2" s="21" t="inlineStr">
+      <c r="G2" s="31" t="inlineStr">
         <is>
           <t>&lt;50M2 (FORFAIT)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>5 cm</t>
         </is>
       </c>
-      <c r="B3" s="23" t="n">
+      <c r="B3" s="33" t="n">
         <v>12.23</v>
       </c>
-      <c r="C3" s="23" t="n">
+      <c r="C3" s="33" t="n">
         <v>12.63</v>
       </c>
-      <c r="D3" s="23" t="n">
+      <c r="D3" s="33" t="n">
         <v>13.03</v>
       </c>
-      <c r="E3" s="23" t="n">
+      <c r="E3" s="33" t="n">
         <v>13.3</v>
       </c>
-      <c r="F3" s="23" t="n">
+      <c r="F3" s="33" t="n">
         <v>13.96</v>
       </c>
-      <c r="G3" s="24" t="n">
+      <c r="G3" s="34" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="32" t="inlineStr">
         <is>
           <t>6 cm</t>
         </is>
       </c>
-      <c r="B4" s="23" t="n">
+      <c r="B4" s="33" t="n">
         <v>13.39</v>
       </c>
-      <c r="C4" s="23" t="n">
+      <c r="C4" s="33" t="n">
         <v>13.83</v>
       </c>
-      <c r="D4" s="23" t="n">
+      <c r="D4" s="33" t="n">
         <v>14.26</v>
       </c>
-      <c r="E4" s="23" t="n">
+      <c r="E4" s="33" t="n">
         <v>14.56</v>
       </c>
-      <c r="F4" s="23" t="n">
+      <c r="F4" s="33" t="n">
         <v>15.28</v>
       </c>
-      <c r="G4" s="24" t="n">
+      <c r="G4" s="34" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>7 cm</t>
         </is>
       </c>
-      <c r="B5" s="23" t="n">
+      <c r="B5" s="33" t="n">
         <v>14.55</v>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="33" t="n">
         <v>15.02</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="33" t="n">
         <v>15.5</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="33" t="n">
         <v>15.82</v>
       </c>
-      <c r="F5" s="23" t="n">
+      <c r="F5" s="33" t="n">
         <v>16.61</v>
       </c>
-      <c r="G5" s="24" t="n">
+      <c r="G5" s="34" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>8 cm</t>
         </is>
       </c>
-      <c r="B6" s="23" t="n">
+      <c r="B6" s="33" t="n">
         <v>15.71</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="33" t="n">
         <v>16.22</v>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="33" t="n">
         <v>16.73</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="33" t="n">
         <v>17.08</v>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="33" t="n">
         <v>17.93</v>
       </c>
-      <c r="G6" s="24" t="n">
+      <c r="G6" s="34" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="32" t="inlineStr">
         <is>
           <t>9 cm</t>
         </is>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="33" t="n">
         <v>16.87</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="33" t="n">
         <v>17.42</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="33" t="n">
         <v>17.97</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="33" t="n">
         <v>18.34</v>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="33" t="n">
         <v>19.25</v>
       </c>
-      <c r="G7" s="24" t="n">
+      <c r="G7" s="34" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="32" t="inlineStr">
         <is>
           <t>10 cm</t>
         </is>
       </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="33" t="n">
         <v>18.03</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="33" t="n">
         <v>18.62</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="33" t="n">
         <v>19.2</v>
       </c>
-      <c r="E8" s="23" t="n">
+      <c r="E8" s="33" t="n">
         <v>19.6</v>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="33" t="n">
         <v>20.58</v>
       </c>
-      <c r="G8" s="24" t="n">
+      <c r="G8" s="34" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>11 cm</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="33" t="n">
         <v>19.19</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="33" t="n">
         <v>19.81</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="33" t="n">
         <v>20.44</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="33" t="n">
         <v>20.86</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="33" t="n">
         <v>21.9</v>
       </c>
-      <c r="G9" s="24" t="n">
+      <c r="G9" s="34" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>12 cm</t>
         </is>
       </c>
-      <c r="B10" s="23" t="n">
+      <c r="B10" s="33" t="n">
         <v>20.35</v>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="33" t="n">
         <v>21.01</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="33" t="n">
         <v>21.67</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="33" t="n">
         <v>22.12</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="33" t="n">
         <v>23.22</v>
       </c>
-      <c r="G10" s="24" t="n">
+      <c r="G10" s="34" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>13 cm</t>
         </is>
       </c>
-      <c r="B11" s="23" t="n">
+      <c r="B11" s="33" t="n">
         <v>21.5</v>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="33" t="n">
         <v>22.21</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="33" t="n">
         <v>22.91</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="33" t="n">
         <v>23.38</v>
       </c>
-      <c r="F11" s="23" t="n">
+      <c r="F11" s="33" t="n">
         <v>24.54</v>
       </c>
-      <c r="G11" s="24" t="n">
+      <c r="G11" s="34" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>14 cm</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="33" t="n">
         <v>22.66</v>
       </c>
-      <c r="C12" s="23" t="n">
+      <c r="C12" s="33" t="n">
         <v>23.4</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="33" t="n">
         <v>24.14</v>
       </c>
-      <c r="E12" s="23" t="n">
+      <c r="E12" s="33" t="n">
         <v>24.64</v>
       </c>
-      <c r="F12" s="23" t="n">
+      <c r="F12" s="33" t="n">
         <v>25.87</v>
       </c>
-      <c r="G12" s="24" t="n">
+      <c r="G12" s="34" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>15 cm</t>
         </is>
       </c>
-      <c r="B13" s="23" t="n">
+      <c r="B13" s="33" t="n">
         <v>23.82</v>
       </c>
-      <c r="C13" s="23" t="n">
+      <c r="C13" s="33" t="n">
         <v>24.6</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="33" t="n">
         <v>25.38</v>
       </c>
-      <c r="E13" s="23" t="n">
+      <c r="E13" s="33" t="n">
         <v>25.9</v>
       </c>
-      <c r="F13" s="23" t="n">
+      <c r="F13" s="33" t="n">
         <v>27.19</v>
       </c>
-      <c r="G13" s="24" t="n">
+      <c r="G13" s="34" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>16 cm</t>
         </is>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="33" t="n">
         <v>24.98</v>
       </c>
-      <c r="C14" s="23" t="n">
+      <c r="C14" s="33" t="n">
         <v>25.8</v>
       </c>
-      <c r="D14" s="23" t="n">
+      <c r="D14" s="33" t="n">
         <v>26.61</v>
       </c>
-      <c r="E14" s="23" t="n">
+      <c r="E14" s="33" t="n">
         <v>27.16</v>
       </c>
-      <c r="F14" s="23" t="n">
+      <c r="F14" s="33" t="n">
         <v>28.51</v>
       </c>
-      <c r="G14" s="24" t="n">
+      <c r="G14" s="34" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>17 cm</t>
         </is>
       </c>
-      <c r="B15" s="23" t="n">
+      <c r="B15" s="33" t="n">
         <v>26.14</v>
       </c>
-      <c r="C15" s="23" t="n">
+      <c r="C15" s="33" t="n">
         <v>26.99</v>
       </c>
-      <c r="D15" s="23" t="n">
+      <c r="D15" s="33" t="n">
         <v>27.85</v>
       </c>
-      <c r="E15" s="23" t="n">
+      <c r="E15" s="33" t="n">
         <v>28.42</v>
       </c>
-      <c r="F15" s="23" t="n">
+      <c r="F15" s="33" t="n">
         <v>29.84</v>
       </c>
-      <c r="G15" s="24" t="n">
+      <c r="G15" s="34" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="32" t="inlineStr">
         <is>
           <t>18 cm</t>
         </is>
       </c>
-      <c r="B16" s="23" t="n">
+      <c r="B16" s="33" t="n">
         <v>27.3</v>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="33" t="n">
         <v>28.19</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="33" t="n">
         <v>29.08</v>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="33" t="n">
         <v>29.68</v>
       </c>
-      <c r="F16" s="23" t="n">
+      <c r="F16" s="33" t="n">
         <v>31.16</v>
       </c>
-      <c r="G16" s="24" t="n">
+      <c r="G16" s="34" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="32" t="inlineStr">
         <is>
           <t>19 cm</t>
         </is>
       </c>
-      <c r="B17" s="23" t="n">
+      <c r="B17" s="33" t="n">
         <v>28.46</v>
       </c>
-      <c r="C17" s="23" t="n">
+      <c r="C17" s="33" t="n">
         <v>29.39</v>
       </c>
-      <c r="D17" s="23" t="n">
+      <c r="D17" s="33" t="n">
         <v>30.32</v>
       </c>
-      <c r="E17" s="23" t="n">
+      <c r="E17" s="33" t="n">
         <v>30.94</v>
       </c>
-      <c r="F17" s="23" t="n">
+      <c r="F17" s="33" t="n">
         <v>32.48</v>
       </c>
-      <c r="G17" s="24" t="n">
+      <c r="G17" s="34" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t>20 cm</t>
         </is>
       </c>
-      <c r="B18" s="23" t="n">
+      <c r="B18" s="33" t="n">
         <v>29.62</v>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="33" t="n">
         <v>30.59</v>
       </c>
-      <c r="D18" s="23" t="n">
+      <c r="D18" s="33" t="n">
         <v>31.55</v>
       </c>
-      <c r="E18" s="23" t="n">
+      <c r="E18" s="33" t="n">
         <v>32.2</v>
       </c>
-      <c r="F18" s="23" t="n">
+      <c r="F18" s="33" t="n">
         <v>33.81</v>
       </c>
-      <c r="G18" s="24" t="n">
+      <c r="G18" s="34" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>21 cm</t>
         </is>
       </c>
-      <c r="B19" s="23" t="n">
+      <c r="B19" s="33" t="n">
         <v>30.78</v>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="33" t="n">
         <v>31.78</v>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="33" t="n">
         <v>32.79</v>
       </c>
-      <c r="E19" s="23" t="n">
+      <c r="E19" s="33" t="n">
         <v>33.46</v>
       </c>
-      <c r="F19" s="23" t="n">
+      <c r="F19" s="33" t="n">
         <v>35.13</v>
       </c>
-      <c r="G19" s="24" t="n">
+      <c r="G19" s="34" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="22" t="inlineStr">
+      <c r="A20" s="32" t="inlineStr">
         <is>
           <t>23 cm</t>
         </is>
       </c>
-      <c r="B20" s="23" t="n">
+      <c r="B20" s="33" t="n">
         <v>33.1</v>
       </c>
-      <c r="C20" s="23" t="n">
+      <c r="C20" s="33" t="n">
         <v>34.18</v>
       </c>
-      <c r="D20" s="23" t="n">
+      <c r="D20" s="33" t="n">
         <v>35.26</v>
       </c>
-      <c r="E20" s="23" t="n">
+      <c r="E20" s="33" t="n">
         <v>35.98</v>
       </c>
-      <c r="F20" s="23" t="n">
+      <c r="F20" s="33" t="n">
         <v>37.77</v>
       </c>
-      <c r="G20" s="24" t="n">
+      <c r="G20" s="34" t="n">
         <v>1800</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="22" t="inlineStr">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t>25 cm</t>
         </is>
       </c>
-      <c r="B21" s="23" t="n">
+      <c r="B21" s="33" t="n">
         <v>35.42</v>
       </c>
-      <c r="C21" s="23" t="n">
+      <c r="C21" s="33" t="n">
         <v>36.57</v>
       </c>
-      <c r="D21" s="23" t="n">
+      <c r="D21" s="33" t="n">
         <v>37.73</v>
       </c>
-      <c r="E21" s="23" t="n">
+      <c r="E21" s="33" t="n">
         <v>38.5</v>
       </c>
-      <c r="F21" s="23" t="n">
+      <c r="F21" s="33" t="n">
         <v>40.42</v>
       </c>
-      <c r="G21" s="24" t="n">
+      <c r="G21" s="34" t="n">
         <v>1800</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Overhaul Excel spreadsheet with side-by-side design layout, huge KPI widget boxes, and slate navy theme
</commit_message>
<xml_diff>
--- a/Calculateur_Mousse_Polyurethane.xlsx
+++ b/Calculateur_Mousse_Polyurethane.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.00 €"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,7 +51,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="20"/>
+      <sz val="22"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -63,7 +63,7 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00334155"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -79,41 +79,50 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <color rgb="00475569"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <sz val="12"/>
+      <color rgb="000369A1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000369A1"/>
+      <sz val="18"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00991B1B"/>
-      <sz val="12"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00991B1B"/>
-      <sz val="13"/>
+      <sz val="18"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="000369A1"/>
+      <color rgb="00166534"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00166534"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00166534"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="000369A1"/>
-      <sz val="13"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -123,18 +132,20 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <color rgb="00475569"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00166534"/>
-      <sz val="15"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00166534"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -149,14 +160,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E293B"/>
-        <bgColor rgb="001E293B"/>
+        <fgColor rgb="000F172A"/>
+        <bgColor rgb="000F172A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00334155"/>
         <bgColor rgb="00334155"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00166534"/>
+        <bgColor rgb="00166534"/>
       </patternFill>
     </fill>
     <fill>
@@ -184,7 +201,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -212,11 +229,145 @@
       </bottom>
     </border>
     <border>
-      <top style="thin">
+      <left style="medium">
+        <color rgb="000369A1"/>
+      </left>
+      <top style="medium">
+        <color rgb="000369A1"/>
+      </top>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="000369A1"/>
+      </top>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="000369A1"/>
+      </right>
+      <top style="medium">
+        <color rgb="000369A1"/>
+      </top>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000369A1"/>
+      </left>
+      <bottom style="medium">
+        <color rgb="000369A1"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="000369A1"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="000369A1"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="000369A1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00991B1B"/>
+      </left>
+      <top style="medium">
+        <color rgb="00991B1B"/>
+      </top>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="00991B1B"/>
+      </top>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="00991B1B"/>
+      </right>
+      <top style="medium">
+        <color rgb="00991B1B"/>
+      </top>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00991B1B"/>
+      </left>
+      <bottom style="medium">
+        <color rgb="00991B1B"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00991B1B"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="00991B1B"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="00991B1B"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00166534"/>
+      </left>
+      <top style="medium">
+        <color rgb="00166534"/>
+      </top>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="00166534"/>
+      </top>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="00166534"/>
+      </right>
+      <top style="medium">
+        <color rgb="00166534"/>
+      </top>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00166534"/>
+      </left>
+      <bottom style="medium">
+        <color rgb="00166534"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="00166534"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
+        <color rgb="00166534"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="00166534"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00166534"/>
+      </left>
+      <bottom style="thin">
         <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="double">
+      </bottom>
+    </border>
+    <border>
+      <right style="medium">
         <color rgb="00166534"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
       </bottom>
     </border>
     <border>
@@ -251,37 +402,14 @@
       <left style="medium">
         <color rgb="00475569"/>
       </left>
-      <top style="medium">
-        <color rgb="00475569"/>
-      </top>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="00475569"/>
-      </left>
       <bottom style="medium">
         <color rgb="00475569"/>
       </bottom>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="00475569"/>
-      </top>
-    </border>
-    <border>
       <bottom style="medium">
         <color rgb="00475569"/>
       </bottom>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="00475569"/>
-      </right>
-      <top style="medium">
-        <color rgb="00475569"/>
-      </top>
     </border>
     <border>
       <right style="medium">
@@ -291,101 +419,104 @@
         <color rgb="00475569"/>
       </bottom>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="00475569"/>
-      </left>
-      <bottom style="double">
-        <color rgb="00166534"/>
-      </bottom>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="00475569"/>
-      </right>
-      <bottom style="double">
-        <color rgb="00166534"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="10" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="12" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="6" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="14" fillId="9" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="17" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="18" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -764,33 +895,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D27"/>
+  <dimension ref="B2:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="55" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Calculateur Mousse Polyuréthane</t>
+          <t>TABLEAU DE BORD DE MARGE POLYURÉTHANE</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1. DONNÉES DU PROJET (SAISIE)</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="4" t="n"/>
-    </row>
-    <row r="5" ht="28" customHeight="1">
+          <t xml:space="preserve"> 🔍 SAISIE DES DONNÉES DU PROJET</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n"/>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 📊 RÉSULTATS FINANCIERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
       <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Surface Totale (Métrage)</t>
@@ -804,14 +942,21 @@
           <t>m²</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="28" customHeight="1">
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>VOTRE FACTURATION CLIENT TOTAL (HT)</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="10" t="n"/>
+    </row>
+    <row r="6" ht="35" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Prix Client au m²</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="11" t="n">
         <v>83.33</v>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -819,6 +964,12 @@
           <t>€/m²</t>
         </is>
       </c>
+      <c r="F6" s="12">
+        <f>C7</f>
+        <v/>
+      </c>
+      <c r="G6" s="13" t="n"/>
+      <c r="H6" s="14" t="n"/>
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="B7" s="5" t="inlineStr">
@@ -826,7 +977,7 @@
           <t>Votre Prix de Vente (Client) Total</t>
         </is>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="11">
         <f>C5*C6</f>
         <v/>
       </c>
@@ -836,13 +987,13 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
+    <row r="8" ht="20" customHeight="1">
       <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Épaisseur de mousse</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>10 cm</t>
         </is>
@@ -852,14 +1003,21 @@
           <t>cm</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>COÛT DU SOUS-TRAITANT TOTAL (HT)</t>
+        </is>
+      </c>
+      <c r="G8" s="17" t="n"/>
+      <c r="H8" s="18" t="n"/>
+    </row>
+    <row r="9" ht="35" customHeight="1">
       <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Distance de Déplacement</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Rayon ≤ 30 Km</t>
         </is>
@@ -869,6 +1027,12 @@
           <t>Choix</t>
         </is>
       </c>
+      <c r="F9" s="19">
+        <f>IF(C5&lt;50, C21, C21*C5)</f>
+        <v/>
+      </c>
+      <c r="G9" s="20" t="n"/>
+      <c r="H9" s="21" t="n"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="B10" s="5" t="inlineStr">
@@ -876,7 +1040,7 @@
           <t>Conditions Partenaire</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
@@ -887,13 +1051,13 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1">
+    <row r="11" ht="20" customHeight="1">
       <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Délai de Paiement</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>30 jours (Standard)</t>
         </is>
@@ -903,178 +1067,158 @@
           <t>Choix</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="B12" s="11" t="inlineStr">
+      <c r="F11" s="22" t="inlineStr">
+        <is>
+          <t>VOTRE BÉNÉFICE NET (DIFFÉRENCE B - A)</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="n"/>
+      <c r="H11" s="24" t="n"/>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="B12" s="25" t="inlineStr">
         <is>
           <t>Majoration Sous-traitant</t>
         </is>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="26" t="n">
         <v>0.1</v>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="27" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
+      <c r="F12" s="28">
+        <f>F6-F9</f>
+        <v/>
+      </c>
+      <c r="G12" s="29" t="n"/>
+      <c r="H12" s="30" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 2. DÉTAILS DU COÛT SOUS-TRAITANT</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="4" t="n"/>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>Catégorie de Surface</t>
-        </is>
-      </c>
-      <c r="C15" s="15">
+          <t xml:space="preserve"> ⚙️ DÉTAILS DE LA FACTURATION SOUS-TRAITANT</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 📈 RENDEMENT &amp; RENTABILITÉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Catégorie de Surface (Calculée)</t>
+        </is>
+      </c>
+      <c r="C15" s="31">
         <f>IF(C5&lt;50, "&lt;50M2 (FORFAIT)", IF(C5&lt;100, "50-100M2 (+5%)", IF(C5&lt;150, "100-150M2 (0%)", IF(C5&lt;250, "150-250M2 (-2%)", IF(C5&lt;=400, "250-400M2 (-5%)", "&gt;400M2 (-8%)")))))</f>
         <v/>
       </c>
-      <c r="D15" s="16" t="inlineStr"/>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="B16" s="14" t="inlineStr">
+      <c r="D15" s="32" t="n"/>
+      <c r="F15" s="33" t="inlineStr">
+        <is>
+          <t>Marge Bénéficiaire (%)</t>
+        </is>
+      </c>
+      <c r="G15" s="34">
+        <f>IF(F6&gt;0, F12/F6, 0)</f>
+        <v/>
+      </c>
+      <c r="H15" s="35" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Tarif de Base NESTAAN</t>
         </is>
       </c>
-      <c r="C16" s="15">
+      <c r="C16" s="36">
         <f>INDEX(Grille!$B$3:$G$21, MATCH(C8, Grille!$A$3:$A$21, 0), MATCH(C15, Grille!$B$2:$G$2, 0))</f>
         <v/>
       </c>
-      <c r="D16" s="16" t="inlineStr"/>
-    </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>Base avec Majoration</t>
-        </is>
-      </c>
-      <c r="C17" s="15">
+      <c r="D16" s="32" t="n"/>
+      <c r="F16" s="37" t="n"/>
+      <c r="G16" s="29" t="n"/>
+      <c r="H16" s="30" t="n"/>
+    </row>
+    <row r="17" ht="25" customHeight="1">
+      <c r="B17" s="38" t="inlineStr">
+        <is>
+          <t>Base avec Majoration (+10%)</t>
+        </is>
+      </c>
+      <c r="C17" s="39">
         <f>C16*(1+C12)</f>
         <v/>
       </c>
-      <c r="D17" s="16" t="inlineStr"/>
-    </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="B18" s="14" t="inlineStr">
+      <c r="D17" s="32" t="n"/>
+    </row>
+    <row r="18" ht="25" customHeight="1">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>Ajustement Rayon / Distance</t>
         </is>
       </c>
-      <c r="C18" s="17">
+      <c r="C18" s="40">
         <f>IF(C9="Rayon de 30 à 60 Km", 1.01, IF(C9="Rayon &gt; 60 Km", 1.02, 1.00))</f>
         <v/>
       </c>
-      <c r="D18" s="16" t="inlineStr"/>
-    </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="B19" s="14" t="inlineStr">
+      <c r="D18" s="32" t="n"/>
+    </row>
+    <row r="19" ht="25" customHeight="1">
+      <c r="B19" s="38" t="inlineStr">
         <is>
           <t>Ajustement Partenaire (-10%)</t>
         </is>
       </c>
-      <c r="C19" s="17">
+      <c r="C19" s="40">
         <f>IF(C10="Oui", 0.90, 1.00)</f>
         <v/>
       </c>
-      <c r="D19" s="16" t="inlineStr"/>
-    </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="B20" s="14" t="inlineStr">
+      <c r="D19" s="32" t="n"/>
+    </row>
+    <row r="20" ht="25" customHeight="1">
+      <c r="B20" s="38" t="inlineStr">
         <is>
           <t>Ajustement Escompte (-2%)</t>
         </is>
       </c>
-      <c r="C20" s="17">
+      <c r="C20" s="40">
         <f>IF(C11="8 jours (-2%)", 0.98, 1.00)</f>
         <v/>
       </c>
-      <c r="D20" s="16" t="inlineStr"/>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="B21" s="11" t="inlineStr">
+      <c r="D20" s="32" t="n"/>
+    </row>
+    <row r="21" ht="25" customHeight="1">
+      <c r="B21" s="25" t="inlineStr">
         <is>
           <t>Tarif Unitaire Final Sous-traitant</t>
         </is>
       </c>
-      <c r="C21" s="18">
+      <c r="C21" s="41">
         <f>C17*C18*C19*C20</f>
         <v/>
       </c>
-      <c r="D21" s="19" t="inlineStr"/>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 3. RÉSULTATS &amp; DIFFÉRENCE (MARGE)</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="4" t="n"/>
-    </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="B24" s="20" t="inlineStr">
-        <is>
-          <t>Coût Sous-traitant (A)</t>
-        </is>
-      </c>
-      <c r="C24" s="21">
-        <f>IF(C5&lt;50, C21, C21*C5)</f>
-        <v/>
-      </c>
-      <c r="D24" s="22" t="n"/>
-    </row>
-    <row r="25" ht="32" customHeight="1">
-      <c r="B25" s="23" t="inlineStr">
-        <is>
-          <t>Votre Facturation Client (B)</t>
-        </is>
-      </c>
-      <c r="C25" s="24">
-        <f>C7</f>
-        <v/>
-      </c>
-      <c r="D25" s="25" t="n"/>
-    </row>
-    <row r="26" ht="38" customHeight="1">
-      <c r="B26" s="26" t="inlineStr">
-        <is>
-          <t>DIFFÉRENCE (Bénéfice B - A)</t>
-        </is>
-      </c>
-      <c r="C26" s="27">
-        <f>C25-C24</f>
-        <v/>
-      </c>
-      <c r="D26" s="28" t="n"/>
-    </row>
-    <row r="27" ht="28" customHeight="1">
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>Marge Bénéficiaire (%)</t>
-        </is>
-      </c>
-      <c r="C27" s="29">
-        <f>IF(C25&gt;0, C26/C25, 0)</f>
-        <v/>
-      </c>
-      <c r="D27" s="19" t="n"/>
+      <c r="D21" s="42" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="B23:D23"/>
+  <mergeCells count="11">
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="F5:H5"/>
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F14:H14"/>
     <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="F12:H12"/>
+    <mergeCell ref="F11:H11"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1113,521 +1257,521 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="30" t="inlineStr">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>Grille de Tarifs NESTAAN S-09 (Hors TVA)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="25" customHeight="1">
-      <c r="A2" s="31" t="inlineStr">
+      <c r="A2" s="44" t="inlineStr">
         <is>
           <t>Épaisseur</t>
         </is>
       </c>
-      <c r="B2" s="31" t="inlineStr">
+      <c r="B2" s="44" t="inlineStr">
         <is>
           <t>&gt;400M2 (-8%)</t>
         </is>
       </c>
-      <c r="C2" s="31" t="inlineStr">
+      <c r="C2" s="44" t="inlineStr">
         <is>
           <t>250-400M2 (-5%)</t>
         </is>
       </c>
-      <c r="D2" s="31" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>150-250M2 (-2%)</t>
         </is>
       </c>
-      <c r="E2" s="31" t="inlineStr">
+      <c r="E2" s="44" t="inlineStr">
         <is>
           <t>100-150M2 (0%)</t>
         </is>
       </c>
-      <c r="F2" s="31" t="inlineStr">
+      <c r="F2" s="44" t="inlineStr">
         <is>
           <t>50-100M2 (+5%)</t>
         </is>
       </c>
-      <c r="G2" s="31" t="inlineStr">
+      <c r="G2" s="44" t="inlineStr">
         <is>
           <t>&lt;50M2 (FORFAIT)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="32" t="inlineStr">
+      <c r="A3" s="45" t="inlineStr">
         <is>
           <t>5 cm</t>
         </is>
       </c>
-      <c r="B3" s="33" t="n">
+      <c r="B3" s="46" t="n">
         <v>12.23</v>
       </c>
-      <c r="C3" s="33" t="n">
+      <c r="C3" s="46" t="n">
         <v>12.63</v>
       </c>
-      <c r="D3" s="33" t="n">
+      <c r="D3" s="46" t="n">
         <v>13.03</v>
       </c>
-      <c r="E3" s="33" t="n">
+      <c r="E3" s="46" t="n">
         <v>13.3</v>
       </c>
-      <c r="F3" s="33" t="n">
+      <c r="F3" s="46" t="n">
         <v>13.96</v>
       </c>
-      <c r="G3" s="34" t="n">
+      <c r="G3" s="47" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="32" t="inlineStr">
+      <c r="A4" s="45" t="inlineStr">
         <is>
           <t>6 cm</t>
         </is>
       </c>
-      <c r="B4" s="33" t="n">
+      <c r="B4" s="46" t="n">
         <v>13.39</v>
       </c>
-      <c r="C4" s="33" t="n">
+      <c r="C4" s="46" t="n">
         <v>13.83</v>
       </c>
-      <c r="D4" s="33" t="n">
+      <c r="D4" s="46" t="n">
         <v>14.26</v>
       </c>
-      <c r="E4" s="33" t="n">
+      <c r="E4" s="46" t="n">
         <v>14.56</v>
       </c>
-      <c r="F4" s="33" t="n">
+      <c r="F4" s="46" t="n">
         <v>15.28</v>
       </c>
-      <c r="G4" s="34" t="n">
+      <c r="G4" s="47" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="32" t="inlineStr">
+      <c r="A5" s="45" t="inlineStr">
         <is>
           <t>7 cm</t>
         </is>
       </c>
-      <c r="B5" s="33" t="n">
+      <c r="B5" s="46" t="n">
         <v>14.55</v>
       </c>
-      <c r="C5" s="33" t="n">
+      <c r="C5" s="46" t="n">
         <v>15.02</v>
       </c>
-      <c r="D5" s="33" t="n">
+      <c r="D5" s="46" t="n">
         <v>15.5</v>
       </c>
-      <c r="E5" s="33" t="n">
+      <c r="E5" s="46" t="n">
         <v>15.82</v>
       </c>
-      <c r="F5" s="33" t="n">
+      <c r="F5" s="46" t="n">
         <v>16.61</v>
       </c>
-      <c r="G5" s="34" t="n">
+      <c r="G5" s="47" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="32" t="inlineStr">
+      <c r="A6" s="45" t="inlineStr">
         <is>
           <t>8 cm</t>
         </is>
       </c>
-      <c r="B6" s="33" t="n">
+      <c r="B6" s="46" t="n">
         <v>15.71</v>
       </c>
-      <c r="C6" s="33" t="n">
+      <c r="C6" s="46" t="n">
         <v>16.22</v>
       </c>
-      <c r="D6" s="33" t="n">
+      <c r="D6" s="46" t="n">
         <v>16.73</v>
       </c>
-      <c r="E6" s="33" t="n">
+      <c r="E6" s="46" t="n">
         <v>17.08</v>
       </c>
-      <c r="F6" s="33" t="n">
+      <c r="F6" s="46" t="n">
         <v>17.93</v>
       </c>
-      <c r="G6" s="34" t="n">
+      <c r="G6" s="47" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="32" t="inlineStr">
+      <c r="A7" s="45" t="inlineStr">
         <is>
           <t>9 cm</t>
         </is>
       </c>
-      <c r="B7" s="33" t="n">
+      <c r="B7" s="46" t="n">
         <v>16.87</v>
       </c>
-      <c r="C7" s="33" t="n">
+      <c r="C7" s="46" t="n">
         <v>17.42</v>
       </c>
-      <c r="D7" s="33" t="n">
+      <c r="D7" s="46" t="n">
         <v>17.97</v>
       </c>
-      <c r="E7" s="33" t="n">
+      <c r="E7" s="46" t="n">
         <v>18.34</v>
       </c>
-      <c r="F7" s="33" t="n">
+      <c r="F7" s="46" t="n">
         <v>19.25</v>
       </c>
-      <c r="G7" s="34" t="n">
+      <c r="G7" s="47" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" s="45" t="inlineStr">
         <is>
           <t>10 cm</t>
         </is>
       </c>
-      <c r="B8" s="33" t="n">
+      <c r="B8" s="46" t="n">
         <v>18.03</v>
       </c>
-      <c r="C8" s="33" t="n">
+      <c r="C8" s="46" t="n">
         <v>18.62</v>
       </c>
-      <c r="D8" s="33" t="n">
+      <c r="D8" s="46" t="n">
         <v>19.2</v>
       </c>
-      <c r="E8" s="33" t="n">
+      <c r="E8" s="46" t="n">
         <v>19.6</v>
       </c>
-      <c r="F8" s="33" t="n">
+      <c r="F8" s="46" t="n">
         <v>20.58</v>
       </c>
-      <c r="G8" s="34" t="n">
+      <c r="G8" s="47" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="A9" s="45" t="inlineStr">
         <is>
           <t>11 cm</t>
         </is>
       </c>
-      <c r="B9" s="33" t="n">
+      <c r="B9" s="46" t="n">
         <v>19.19</v>
       </c>
-      <c r="C9" s="33" t="n">
+      <c r="C9" s="46" t="n">
         <v>19.81</v>
       </c>
-      <c r="D9" s="33" t="n">
+      <c r="D9" s="46" t="n">
         <v>20.44</v>
       </c>
-      <c r="E9" s="33" t="n">
+      <c r="E9" s="46" t="n">
         <v>20.86</v>
       </c>
-      <c r="F9" s="33" t="n">
+      <c r="F9" s="46" t="n">
         <v>21.9</v>
       </c>
-      <c r="G9" s="34" t="n">
+      <c r="G9" s="47" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="45" t="inlineStr">
         <is>
           <t>12 cm</t>
         </is>
       </c>
-      <c r="B10" s="33" t="n">
+      <c r="B10" s="46" t="n">
         <v>20.35</v>
       </c>
-      <c r="C10" s="33" t="n">
+      <c r="C10" s="46" t="n">
         <v>21.01</v>
       </c>
-      <c r="D10" s="33" t="n">
+      <c r="D10" s="46" t="n">
         <v>21.67</v>
       </c>
-      <c r="E10" s="33" t="n">
+      <c r="E10" s="46" t="n">
         <v>22.12</v>
       </c>
-      <c r="F10" s="33" t="n">
+      <c r="F10" s="46" t="n">
         <v>23.22</v>
       </c>
-      <c r="G10" s="34" t="n">
+      <c r="G10" s="47" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="32" t="inlineStr">
+      <c r="A11" s="45" t="inlineStr">
         <is>
           <t>13 cm</t>
         </is>
       </c>
-      <c r="B11" s="33" t="n">
+      <c r="B11" s="46" t="n">
         <v>21.5</v>
       </c>
-      <c r="C11" s="33" t="n">
+      <c r="C11" s="46" t="n">
         <v>22.21</v>
       </c>
-      <c r="D11" s="33" t="n">
+      <c r="D11" s="46" t="n">
         <v>22.91</v>
       </c>
-      <c r="E11" s="33" t="n">
+      <c r="E11" s="46" t="n">
         <v>23.38</v>
       </c>
-      <c r="F11" s="33" t="n">
+      <c r="F11" s="46" t="n">
         <v>24.54</v>
       </c>
-      <c r="G11" s="34" t="n">
+      <c r="G11" s="47" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="45" t="inlineStr">
         <is>
           <t>14 cm</t>
         </is>
       </c>
-      <c r="B12" s="33" t="n">
+      <c r="B12" s="46" t="n">
         <v>22.66</v>
       </c>
-      <c r="C12" s="33" t="n">
+      <c r="C12" s="46" t="n">
         <v>23.4</v>
       </c>
-      <c r="D12" s="33" t="n">
+      <c r="D12" s="46" t="n">
         <v>24.14</v>
       </c>
-      <c r="E12" s="33" t="n">
+      <c r="E12" s="46" t="n">
         <v>24.64</v>
       </c>
-      <c r="F12" s="33" t="n">
+      <c r="F12" s="46" t="n">
         <v>25.87</v>
       </c>
-      <c r="G12" s="34" t="n">
+      <c r="G12" s="47" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="A13" s="45" t="inlineStr">
         <is>
           <t>15 cm</t>
         </is>
       </c>
-      <c r="B13" s="33" t="n">
+      <c r="B13" s="46" t="n">
         <v>23.82</v>
       </c>
-      <c r="C13" s="33" t="n">
+      <c r="C13" s="46" t="n">
         <v>24.6</v>
       </c>
-      <c r="D13" s="33" t="n">
+      <c r="D13" s="46" t="n">
         <v>25.38</v>
       </c>
-      <c r="E13" s="33" t="n">
+      <c r="E13" s="46" t="n">
         <v>25.9</v>
       </c>
-      <c r="F13" s="33" t="n">
+      <c r="F13" s="46" t="n">
         <v>27.19</v>
       </c>
-      <c r="G13" s="34" t="n">
+      <c r="G13" s="47" t="n">
         <v>1400</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="45" t="inlineStr">
         <is>
           <t>16 cm</t>
         </is>
       </c>
-      <c r="B14" s="33" t="n">
+      <c r="B14" s="46" t="n">
         <v>24.98</v>
       </c>
-      <c r="C14" s="33" t="n">
+      <c r="C14" s="46" t="n">
         <v>25.8</v>
       </c>
-      <c r="D14" s="33" t="n">
+      <c r="D14" s="46" t="n">
         <v>26.61</v>
       </c>
-      <c r="E14" s="33" t="n">
+      <c r="E14" s="46" t="n">
         <v>27.16</v>
       </c>
-      <c r="F14" s="33" t="n">
+      <c r="F14" s="46" t="n">
         <v>28.51</v>
       </c>
-      <c r="G14" s="34" t="n">
+      <c r="G14" s="47" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="32" t="inlineStr">
+      <c r="A15" s="45" t="inlineStr">
         <is>
           <t>17 cm</t>
         </is>
       </c>
-      <c r="B15" s="33" t="n">
+      <c r="B15" s="46" t="n">
         <v>26.14</v>
       </c>
-      <c r="C15" s="33" t="n">
+      <c r="C15" s="46" t="n">
         <v>26.99</v>
       </c>
-      <c r="D15" s="33" t="n">
+      <c r="D15" s="46" t="n">
         <v>27.85</v>
       </c>
-      <c r="E15" s="33" t="n">
+      <c r="E15" s="46" t="n">
         <v>28.42</v>
       </c>
-      <c r="F15" s="33" t="n">
+      <c r="F15" s="46" t="n">
         <v>29.84</v>
       </c>
-      <c r="G15" s="34" t="n">
+      <c r="G15" s="47" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="A16" s="45" t="inlineStr">
         <is>
           <t>18 cm</t>
         </is>
       </c>
-      <c r="B16" s="33" t="n">
+      <c r="B16" s="46" t="n">
         <v>27.3</v>
       </c>
-      <c r="C16" s="33" t="n">
+      <c r="C16" s="46" t="n">
         <v>28.19</v>
       </c>
-      <c r="D16" s="33" t="n">
+      <c r="D16" s="46" t="n">
         <v>29.08</v>
       </c>
-      <c r="E16" s="33" t="n">
+      <c r="E16" s="46" t="n">
         <v>29.68</v>
       </c>
-      <c r="F16" s="33" t="n">
+      <c r="F16" s="46" t="n">
         <v>31.16</v>
       </c>
-      <c r="G16" s="34" t="n">
+      <c r="G16" s="47" t="n">
         <v>1500</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="32" t="inlineStr">
+      <c r="A17" s="45" t="inlineStr">
         <is>
           <t>19 cm</t>
         </is>
       </c>
-      <c r="B17" s="33" t="n">
+      <c r="B17" s="46" t="n">
         <v>28.46</v>
       </c>
-      <c r="C17" s="33" t="n">
+      <c r="C17" s="46" t="n">
         <v>29.39</v>
       </c>
-      <c r="D17" s="33" t="n">
+      <c r="D17" s="46" t="n">
         <v>30.32</v>
       </c>
-      <c r="E17" s="33" t="n">
+      <c r="E17" s="46" t="n">
         <v>30.94</v>
       </c>
-      <c r="F17" s="33" t="n">
+      <c r="F17" s="46" t="n">
         <v>32.48</v>
       </c>
-      <c r="G17" s="34" t="n">
+      <c r="G17" s="47" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="45" t="inlineStr">
         <is>
           <t>20 cm</t>
         </is>
       </c>
-      <c r="B18" s="33" t="n">
+      <c r="B18" s="46" t="n">
         <v>29.62</v>
       </c>
-      <c r="C18" s="33" t="n">
+      <c r="C18" s="46" t="n">
         <v>30.59</v>
       </c>
-      <c r="D18" s="33" t="n">
+      <c r="D18" s="46" t="n">
         <v>31.55</v>
       </c>
-      <c r="E18" s="33" t="n">
+      <c r="E18" s="46" t="n">
         <v>32.2</v>
       </c>
-      <c r="F18" s="33" t="n">
+      <c r="F18" s="46" t="n">
         <v>33.81</v>
       </c>
-      <c r="G18" s="34" t="n">
+      <c r="G18" s="47" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A19" s="45" t="inlineStr">
         <is>
           <t>21 cm</t>
         </is>
       </c>
-      <c r="B19" s="33" t="n">
+      <c r="B19" s="46" t="n">
         <v>30.78</v>
       </c>
-      <c r="C19" s="33" t="n">
+      <c r="C19" s="46" t="n">
         <v>31.78</v>
       </c>
-      <c r="D19" s="33" t="n">
+      <c r="D19" s="46" t="n">
         <v>32.79</v>
       </c>
-      <c r="E19" s="33" t="n">
+      <c r="E19" s="46" t="n">
         <v>33.46</v>
       </c>
-      <c r="F19" s="33" t="n">
+      <c r="F19" s="46" t="n">
         <v>35.13</v>
       </c>
-      <c r="G19" s="34" t="n">
+      <c r="G19" s="47" t="n">
         <v>1600</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="45" t="inlineStr">
         <is>
           <t>23 cm</t>
         </is>
       </c>
-      <c r="B20" s="33" t="n">
+      <c r="B20" s="46" t="n">
         <v>33.1</v>
       </c>
-      <c r="C20" s="33" t="n">
+      <c r="C20" s="46" t="n">
         <v>34.18</v>
       </c>
-      <c r="D20" s="33" t="n">
+      <c r="D20" s="46" t="n">
         <v>35.26</v>
       </c>
-      <c r="E20" s="33" t="n">
+      <c r="E20" s="46" t="n">
         <v>35.98</v>
       </c>
-      <c r="F20" s="33" t="n">
+      <c r="F20" s="46" t="n">
         <v>37.77</v>
       </c>
-      <c r="G20" s="34" t="n">
+      <c r="G20" s="47" t="n">
         <v>1800</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="45" t="inlineStr">
         <is>
           <t>25 cm</t>
         </is>
       </c>
-      <c r="B21" s="33" t="n">
+      <c r="B21" s="46" t="n">
         <v>35.42</v>
       </c>
-      <c r="C21" s="33" t="n">
+      <c r="C21" s="46" t="n">
         <v>36.57</v>
       </c>
-      <c r="D21" s="33" t="n">
+      <c r="D21" s="46" t="n">
         <v>37.73</v>
       </c>
-      <c r="E21" s="33" t="n">
+      <c r="E21" s="46" t="n">
         <v>38.5</v>
       </c>
-      <c r="F21" s="33" t="n">
+      <c r="F21" s="46" t="n">
         <v>40.42</v>
       </c>
-      <c r="G21" s="34" t="n">
+      <c r="G21" s="47" t="n">
         <v>1800</v>
       </c>
     </row>

</xml_diff>